<commit_message>
Update adv py topics
</commit_message>
<xml_diff>
--- a/p/py-25/topic-list.xlsx
+++ b/p/py-25/topic-list.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12200" tabRatio="698" firstSheet="1" activeTab="2"/>
+    <workbookView windowWidth="28800" windowHeight="12200" tabRatio="698" firstSheet="1" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="core" sheetId="2" r:id="rId1"/>
@@ -15,13 +15,13 @@
     <sheet name="async" sheetId="5" r:id="rId6"/>
     <sheet name="py-ques" sheetId="6" r:id="rId7"/>
     <sheet name="-" sheetId="8" r:id="rId8"/>
-    <sheet name="UT" sheetId="4" r:id="rId9"/>
-    <sheet name="--" sheetId="11" r:id="rId10"/>
-    <sheet name="pandas" sheetId="7" r:id="rId11"/>
-    <sheet name=".." sheetId="12" r:id="rId12"/>
-    <sheet name="Flask" sheetId="10" r:id="rId13"/>
-    <sheet name="." sheetId="14" r:id="rId14"/>
-    <sheet name="py-db" sheetId="13" r:id="rId15"/>
+    <sheet name="pandas" sheetId="7" r:id="rId9"/>
+    <sheet name=".." sheetId="12" r:id="rId10"/>
+    <sheet name="Flask" sheetId="10" r:id="rId11"/>
+    <sheet name="." sheetId="14" r:id="rId12"/>
+    <sheet name="py-db" sheetId="13" r:id="rId13"/>
+    <sheet name="--" sheetId="11" r:id="rId14"/>
+    <sheet name="UT" sheetId="4" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="342">
   <si>
     <t>Most basic things in py</t>
   </si>
@@ -136,6 +136,9 @@
     <t>type dict</t>
   </si>
   <si>
+    <t>Basics 706 Generator</t>
+  </si>
+  <si>
     <t>generator function</t>
   </si>
   <si>
@@ -190,6 +193,30 @@
     <t>objects</t>
   </si>
   <si>
+    <t>__code__</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Ellipisis or ...</t>
+  </si>
+  <si>
+    <t>for slicings</t>
+  </si>
+  <si>
+    <t>NotImplemented</t>
+  </si>
+  <si>
+    <t>Internal Objects</t>
+  </si>
+  <si>
+    <t>contextmanager</t>
+  </si>
+  <si>
+    <t>__enter__ __exit__</t>
+  </si>
+  <si>
     <t>decorators</t>
   </si>
   <si>
@@ -218,29 +245,23 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
       <t xml:space="preserve">print(b, </t>
     </r>
     <r>
       <rPr>
         <b/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
+        <rFont val="Bahnschrift"/>
         <charset val="134"/>
       </rPr>
       <t>end = ', ', flush = True</t>
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
+        <sz val="10"/>
         <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
+        <rFont val="Bahnschrift"/>
         <charset val="134"/>
       </rPr>
       <t>)</t>
@@ -307,6 +328,15 @@
     <t>ipdb set trace</t>
   </si>
   <si>
+    <t>https://docs.python.org/3/library/stdtypes.html#binary-sequence-types-bytes-bytearray-memoryview</t>
+  </si>
+  <si>
+    <t>bytes</t>
+  </si>
+  <si>
+    <t>The principal built-in types are numerics, sequences, mappings, classes, instances and exceptions</t>
+  </si>
+  <si>
     <t>Working with data types built-in functions</t>
   </si>
   <si>
@@ -364,6 +394,12 @@
     <t>integer</t>
   </si>
   <si>
+    <t>https://docs.python.org/3/library/stdtypes.html#integer-string-conversion-length-limitation</t>
+  </si>
+  <si>
+    <t>int('1' * 500_000) can take over 1 sec for compute on fast CPU</t>
+  </si>
+  <si>
     <t>set</t>
   </si>
   <si>
@@ -391,6 +427,45 @@
     <t>reverse string [::-1]</t>
   </si>
   <si>
+    <t>startswith</t>
+  </si>
+  <si>
+    <t>Basics 102 Basic string operations</t>
+  </si>
+  <si>
+    <t>isalnum, isalpha, isnumeric</t>
+  </si>
+  <si>
+    <t>endswith, find, rfind, replace, count</t>
+  </si>
+  <si>
+    <t>string.ascii_letters</t>
+  </si>
+  <si>
+    <t>pre-defined constants</t>
+  </si>
+  <si>
+    <t>Basics 104 String manipulate</t>
+  </si>
+  <si>
+    <t>rjust, center, ljust, maketrans</t>
+  </si>
+  <si>
+    <t>.digits, .hexdigits, .punctuation</t>
+  </si>
+  <si>
+    <t>translate</t>
+  </si>
+  <si>
+    <t>Basics 105 String formating</t>
+  </si>
+  <si>
+    <t>template</t>
+  </si>
+  <si>
+    <t>.substitute</t>
+  </si>
+  <si>
     <t>formattings</t>
   </si>
   <si>
@@ -427,6 +502,24 @@
     <t>comprehensions</t>
   </si>
   <si>
+    <t>Basics 206 Sort Bisect</t>
+  </si>
+  <si>
+    <t>bisect</t>
+  </si>
+  <si>
+    <t>bisect, bisect_right, bisect_left, insort_right, insort_left</t>
+  </si>
+  <si>
+    <t>Basics 205 Sort Efficient using array</t>
+  </si>
+  <si>
+    <t>array</t>
+  </si>
+  <si>
+    <t>insert, append, extend. tolist, getsizeof</t>
+  </si>
+  <si>
     <t>tuple</t>
   </si>
   <si>
@@ -448,6 +541,60 @@
     <t>map lambda</t>
   </si>
   <si>
+    <t>Advance and less used things in py</t>
+  </si>
+  <si>
+    <t>Basics 301 Magic Methods</t>
+  </si>
+  <si>
+    <t>magic method</t>
+  </si>
+  <si>
+    <t>dunder methods</t>
+  </si>
+  <si>
+    <t>__str, __repr, __eq, __ge, __lt, __getattribute, __setattr, __getattr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">__call, __init, </t>
+  </si>
+  <si>
+    <t>Adv 301 function documentation</t>
+  </si>
+  <si>
+    <t>__doc__</t>
+  </si>
+  <si>
+    <t>Basics 401 Define Data Class</t>
+  </si>
+  <si>
+    <t>dataclass</t>
+  </si>
+  <si>
+    <t>Basics 402 Using Post initialization</t>
+  </si>
+  <si>
+    <t>__post_init</t>
+  </si>
+  <si>
+    <t>default value attributes</t>
+  </si>
+  <si>
+    <t>Basics 403 Using default values</t>
+  </si>
+  <si>
+    <t>field</t>
+  </si>
+  <si>
+    <t>frozen</t>
+  </si>
+  <si>
+    <t>dataclasses.FrozenInstanceError</t>
+  </si>
+  <si>
+    <t>context</t>
+  </si>
+  <si>
     <t>Other iteration methods</t>
   </si>
   <si>
@@ -463,61 +610,94 @@
     <t>reverse=True</t>
   </si>
   <si>
+    <t>Basics 202 sorting with key params</t>
+  </si>
+  <si>
     <t>key</t>
   </si>
   <si>
+    <t>Basics 204 Sort Operators</t>
+  </si>
+  <si>
+    <t>itemgetter</t>
+  </si>
+  <si>
+    <t>operators, attrgetter, methodcaller</t>
+  </si>
+  <si>
     <t>enumerate</t>
   </si>
   <si>
+    <t>Adv 201 Utilities    202 Iterator</t>
+  </si>
+  <si>
+    <t>any</t>
+  </si>
+  <si>
     <t>Container methods</t>
   </si>
   <si>
     <t>len, reversed, list, sum, max, min, any, all, zip</t>
   </si>
   <si>
-    <t>Advance and less used things in py</t>
-  </si>
-  <si>
-    <t>Basics 301 Magic Methods</t>
-  </si>
-  <si>
-    <t>magic method</t>
-  </si>
-  <si>
-    <t>dunder methods</t>
-  </si>
-  <si>
-    <t>__str, __repr, __eq, __ge, __lt, __getattribute, __setattr, __getattr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">__call, __init, </t>
-  </si>
-  <si>
-    <t>Basics 401 Define Data Class</t>
-  </si>
-  <si>
-    <t>dataclass</t>
-  </si>
-  <si>
-    <t>Basics 402 Using Post initialization</t>
-  </si>
-  <si>
-    <t>__post_init</t>
-  </si>
-  <si>
-    <t>default value attributes</t>
-  </si>
-  <si>
-    <t>Basics 403 Using default values</t>
-  </si>
-  <si>
-    <t>field</t>
-  </si>
-  <si>
-    <t>frozen</t>
-  </si>
-  <si>
-    <t>dataclasses.FrozenInstanceError</t>
+    <t>Adv 203 Transform</t>
+  </si>
+  <si>
+    <t>filter, map</t>
+  </si>
+  <si>
+    <t>Adv 204 Itertools and lambda</t>
+  </si>
+  <si>
+    <t>itertools</t>
+  </si>
+  <si>
+    <t>count, accumulate, dropwhile, takewhile, cycle</t>
+  </si>
+  <si>
+    <t>Adv 304 Keyword only arguments</t>
+  </si>
+  <si>
+    <t>suppressExceptions=False</t>
+  </si>
+  <si>
+    <t>Adv 402 namedtuple</t>
+  </si>
+  <si>
+    <t>Adv 403 defaultdict</t>
+  </si>
+  <si>
+    <t>Adv 405 Ordered dict</t>
+  </si>
+  <si>
+    <t>Adv 404 Counters</t>
+  </si>
+  <si>
+    <t>values, subtract, update, most_common(3)</t>
+  </si>
+  <si>
+    <t>Adv 406 Deque Objects</t>
+  </si>
+  <si>
+    <t>pop, popleft, append</t>
+  </si>
+  <si>
+    <t>deque</t>
+  </si>
+  <si>
+    <t>rotate, appendleft</t>
+  </si>
+  <si>
+    <t>Adv 502 Enumeration class</t>
+  </si>
+  <si>
+    <t>Enum, unique, auto</t>
+  </si>
+  <si>
+    <t>from enum</t>
+  </si>
+  <si>
+    <t>@unique</t>
   </si>
   <si>
     <t>Common modules which can be used anywhere</t>
@@ -550,18 +730,105 @@
     <t>ZeroDivisionError</t>
   </si>
   <si>
+    <t>URLError</t>
+  </si>
+  <si>
+    <t>HTTPError</t>
+  </si>
+  <si>
+    <t>Basics 601 Working with URLs</t>
+  </si>
+  <si>
+    <t>urllib</t>
+  </si>
+  <si>
+    <t>.parse.urlparse(uurl)</t>
+  </si>
+  <si>
+    <t>.request</t>
+  </si>
+  <si>
+    <t>Basics 302 Basic Requests</t>
+  </si>
+  <si>
+    <t>request</t>
+  </si>
+  <si>
+    <t>Extr 302 Send data - retrieve</t>
+  </si>
+  <si>
+    <t>set http method</t>
+  </si>
+  <si>
+    <t>set headers, body data</t>
+  </si>
+  <si>
+    <t>response parsing</t>
+  </si>
+  <si>
+    <t>using auth</t>
+  </si>
+  <si>
+    <t>Basics 304 Using Authentication</t>
+  </si>
+  <si>
+    <t>HTTPDigestAuth</t>
+  </si>
+  <si>
+    <t>Basics 305 Advanced features</t>
+  </si>
+  <si>
+    <t>timeout, debug redirects</t>
+  </si>
+  <si>
+    <t>user-agent</t>
+  </si>
+  <si>
+    <t>.session</t>
+  </si>
+  <si>
+    <t>Extr 303 Request error handling</t>
+  </si>
+  <si>
+    <t>Errors, Timeout, HTTPError</t>
+  </si>
+  <si>
+    <t>result.raise_for_status()</t>
+  </si>
+  <si>
     <t>random</t>
   </si>
   <si>
+    <t>Basics 203 random</t>
+  </si>
+  <si>
     <t>choice</t>
   </si>
   <si>
     <t>randint</t>
   </si>
   <si>
+    <t>sample</t>
+  </si>
+  <si>
     <t>shuffle</t>
   </si>
   <si>
+    <t>randrange</t>
+  </si>
+  <si>
+    <t>Basics 401 random numbers</t>
+  </si>
+  <si>
+    <t>seed</t>
+  </si>
+  <si>
+    <t>random.random</t>
+  </si>
+  <si>
+    <t>uniform</t>
+  </si>
+  <si>
     <t>datetime</t>
   </si>
   <si>
@@ -604,6 +871,12 @@
     <t>path.getmtime</t>
   </si>
   <si>
+    <t>Basics 304 File seeking</t>
+  </si>
+  <si>
+    <t>seeking</t>
+  </si>
+  <si>
     <t>os</t>
   </si>
   <si>
@@ -619,46 +892,139 @@
     <t>getcwd, urandom</t>
   </si>
   <si>
+    <t>Basics 403 cryptographical secure</t>
+  </si>
+  <si>
+    <t>cryptographical secure</t>
+  </si>
+  <si>
+    <t>secrets</t>
+  </si>
+  <si>
+    <t>token-urlsafe</t>
+  </si>
+  <si>
+    <t>choice, token_bytes, token_hex</t>
+  </si>
+  <si>
+    <t>Basics 404 Temporary password</t>
+  </si>
+  <si>
+    <t>create temp password with rules</t>
+  </si>
+  <si>
     <t>copy</t>
   </si>
   <si>
     <t>shallow copy, deepcopy</t>
   </si>
   <si>
+    <t>Basics 205 Iterators with itertools</t>
+  </si>
+  <si>
+    <t>count, cycle, repeat</t>
+  </si>
+  <si>
+    <t>permutations, combinatins</t>
+  </si>
+  <si>
+    <t>csv</t>
+  </si>
+  <si>
+    <t>reader, read, Sniffer().sniff</t>
+  </si>
+  <si>
+    <t>reader</t>
+  </si>
+  <si>
+    <t>csv.Sniffer().has_header, .writter, writerow</t>
+  </si>
+  <si>
+    <t>json</t>
+  </si>
+  <si>
+    <t>loads</t>
+  </si>
+  <si>
+    <t>null value</t>
+  </si>
+  <si>
+    <t>Basics 604 JSON</t>
+  </si>
+  <si>
+    <t>dumps</t>
+  </si>
+  <si>
+    <t>Extr 401 JSON Module</t>
+  </si>
+  <si>
+    <t>load vs loads</t>
+  </si>
+  <si>
+    <t>dump vs dumps</t>
+  </si>
+  <si>
+    <t>what js datatype will covert to what via this module</t>
+  </si>
+  <si>
+    <t>JSONDecodeError</t>
+  </si>
+  <si>
+    <t>xml</t>
+  </si>
+  <si>
+    <t>nodeName</t>
+  </si>
+  <si>
+    <t>firstChild.tagName</t>
+  </si>
+  <si>
+    <t>setAttribute</t>
+  </si>
+  <si>
+    <t>createElement</t>
+  </si>
+  <si>
+    <t>Basics 306 Configuration files</t>
+  </si>
+  <si>
+    <t>configparser</t>
+  </si>
+  <si>
+    <t>read, sections, has_sections</t>
+  </si>
+  <si>
+    <t>.ConfigParser()</t>
+  </si>
+  <si>
+    <t>Basics 405 Unique Identifier</t>
+  </si>
+  <si>
+    <t>uuid</t>
+  </si>
+  <si>
+    <t>uuid4(), uuid5()</t>
+  </si>
+  <si>
+    <t>feature rich xml and html</t>
+  </si>
+  <si>
+    <t>lxml</t>
+  </si>
+  <si>
     <t>shutil</t>
   </si>
   <si>
+    <t>Basics 307 Manipulate zip files</t>
+  </si>
+  <si>
     <t>zipfile</t>
   </si>
   <si>
-    <t>urllib</t>
-  </si>
-  <si>
-    <t>json</t>
-  </si>
-  <si>
-    <t>loads</t>
-  </si>
-  <si>
-    <t>null value</t>
-  </si>
-  <si>
-    <t>dumps</t>
-  </si>
-  <si>
-    <t>xml</t>
-  </si>
-  <si>
-    <t>nodeName</t>
-  </si>
-  <si>
-    <t>firstChild.tagName</t>
-  </si>
-  <si>
-    <t>setAttribute</t>
-  </si>
-  <si>
-    <t>createElement</t>
+    <t>ZipFile, namelist, infolist, getinfo, open</t>
+  </si>
+  <si>
+    <t>extract, extractall, close</t>
   </si>
   <si>
     <t>Basics 201 Pendulum - datetime</t>
@@ -676,37 +1042,22 @@
     <t>debugger</t>
   </si>
   <si>
-    <t>Basics 302 Basic Requests</t>
-  </si>
-  <si>
-    <t>request</t>
-  </si>
-  <si>
-    <t>set http method</t>
-  </si>
-  <si>
-    <t>set headers, body data</t>
-  </si>
-  <si>
-    <t>response parsing</t>
-  </si>
-  <si>
-    <t>using auth</t>
-  </si>
-  <si>
-    <t>Basics 304 Using Authentication</t>
-  </si>
-  <si>
-    <t>HTTPDigestAuth</t>
-  </si>
-  <si>
-    <t>Basics 305 Advanced features</t>
-  </si>
-  <si>
-    <t>timeout, debug redirects</t>
-  </si>
-  <si>
-    <t>user-agent</t>
+    <t>Basics 204 Statistics</t>
+  </si>
+  <si>
+    <t>statistics</t>
+  </si>
+  <si>
+    <t>mean, mode, median</t>
+  </si>
+  <si>
+    <t>variance, stdev</t>
+  </si>
+  <si>
+    <t>Basics 406 Text Wrap</t>
+  </si>
+  <si>
+    <t>textwrap</t>
   </si>
   <si>
     <t>fibonacci</t>
@@ -727,10 +1078,16 @@
     <t>n%x === 0: return false</t>
   </si>
   <si>
-    <t>format str</t>
-  </si>
-  <si>
     <t>how id works</t>
+  </si>
+  <si>
+    <t>anagrams</t>
+  </si>
+  <si>
+    <t>find possible words of given character</t>
+  </si>
+  <si>
+    <t>httpbin test</t>
   </si>
 </sst>
 </file>
@@ -743,7 +1100,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="30">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -769,9 +1126,16 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
+      <i/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Bahnschrift"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
+      <name val="Bahnschrift"/>
       <charset val="134"/>
     </font>
     <font>
@@ -783,9 +1147,16 @@
       <charset val="134"/>
     </font>
     <font>
+      <u/>
       <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Bahnschrift"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Bahnschrift"/>
+      <name val="Calibri"/>
       <charset val="134"/>
     </font>
     <font>
@@ -941,9 +1312,9 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
+      <name val="Bahnschrift"/>
       <charset val="134"/>
     </font>
   </fonts>
@@ -1250,28 +1621,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1280,143 +1642,165 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1756,7 +2140,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="12.5" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="27.3307692307692" style="1" customWidth="1"/>
@@ -1787,7 +2171,7 @@
       <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="5" t="s">
         <v>5</v>
       </c>
       <c r="H2" s="1" t="s">
@@ -1798,22 +2182,22 @@
       <c r="C3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="2"/>
+      <c r="G3" s="5"/>
     </row>
     <row r="4" spans="4:7">
       <c r="D4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="2"/>
+      <c r="G4" s="5"/>
     </row>
     <row r="5" spans="4:7">
       <c r="D5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="2"/>
+      <c r="G5" s="5"/>
     </row>
     <row r="6" spans="7:7">
-      <c r="G6" s="2"/>
+      <c r="G6" s="5"/>
     </row>
     <row r="7" spans="3:3">
       <c r="C7" s="1" t="s">
@@ -1846,16 +2230,16 @@
       </c>
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:8">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
     </row>
     <row r="16" spans="3:3">
       <c r="C16" s="1" t="s">
@@ -1878,12 +2262,12 @@
       </c>
     </row>
     <row r="21" spans="4:4">
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="12" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="22" spans="4:5">
-      <c r="D22" s="7"/>
+      <c r="D22" s="12"/>
       <c r="E22" s="1" t="s">
         <v>22</v>
       </c>
@@ -1920,129 +2304,148 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="3:6">
+    <row r="28" spans="1:6">
+      <c r="A28" s="1" t="s">
+        <v>31</v>
+      </c>
       <c r="C28" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="30" spans="3:3">
       <c r="C30" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="31" spans="2:4">
       <c r="B31" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="32" spans="4:4">
       <c r="D32" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="33" spans="1:4">
-      <c r="A33" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="B33" s="12"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="12" t="s">
+      <c r="A33" s="19" t="s">
         <v>38</v>
       </c>
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="34" spans="1:4">
-      <c r="A34" s="12" t="s">
-        <v>39</v>
+      <c r="A34" s="19" t="s">
+        <v>40</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="35" spans="1:4">
-      <c r="A35" s="12" t="s">
-        <v>41</v>
+      <c r="A35" s="19" t="s">
+        <v>42</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="36" spans="1:1">
-      <c r="A36" s="12"/>
+      <c r="A36" s="19"/>
     </row>
     <row r="37" spans="3:3">
       <c r="C37" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" s="12" t="s">
-        <v>44</v>
+      <c r="A38" s="19" t="s">
+        <v>45</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39" spans="3:3">
       <c r="C39" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="41" spans="3:3">
       <c r="C41" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="43" ht="15.5" spans="1:3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="42" spans="4:4">
+      <c r="D42" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="43" ht="15.5" spans="1:4">
       <c r="A43"/>
       <c r="B43"/>
       <c r="C43"/>
-    </row>
-    <row r="45" spans="3:3">
-      <c r="C45" s="1" t="s">
-        <v>49</v>
+      <c r="D43" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="44" spans="4:6">
+      <c r="D44" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="45" spans="4:4">
+      <c r="D45" s="1" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="46" spans="4:4">
       <c r="D46" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4">
-      <c r="A47" s="1" t="s">
-        <v>51</v>
-      </c>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="47" spans="4:4">
       <c r="D47" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="49" ht="15.5" spans="3:5">
-      <c r="C49"/>
-      <c r="D49"/>
-      <c r="E49"/>
-    </row>
-    <row r="50" ht="15.5" spans="3:5">
-      <c r="C50"/>
-      <c r="D50"/>
-      <c r="E50"/>
-    </row>
-    <row r="51" ht="15.5" spans="3:5">
-      <c r="C51"/>
-      <c r="D51"/>
-      <c r="E51"/>
-    </row>
-    <row r="52" ht="15.5" spans="3:5">
-      <c r="C52"/>
-      <c r="D52"/>
-      <c r="E52"/>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="48" spans="5:5">
+      <c r="E48" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="49" spans="3:3">
+      <c r="C49" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="50" spans="4:4">
+      <c r="D50" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="A51" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="53" ht="15.5" spans="3:5">
       <c r="C53"/>
@@ -2078,6 +2481,26 @@
       <c r="C59"/>
       <c r="D59"/>
       <c r="E59"/>
+    </row>
+    <row r="60" ht="15.5" spans="3:5">
+      <c r="C60"/>
+      <c r="D60"/>
+      <c r="E60"/>
+    </row>
+    <row r="61" ht="15.5" spans="3:5">
+      <c r="C61"/>
+      <c r="D61"/>
+      <c r="E61"/>
+    </row>
+    <row r="62" ht="15.5" spans="3:5">
+      <c r="C62"/>
+      <c r="D62"/>
+      <c r="E62"/>
+    </row>
+    <row r="63" ht="15.5" spans="3:5">
+      <c r="C63"/>
+      <c r="D63"/>
+      <c r="E63"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2134,13 +2557,43 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.66923076923077" defaultRowHeight="12.5"/>
+  <dimension ref="A2:H2"/>
+  <sheetFormatPr defaultColWidth="8.66923076923077" defaultRowHeight="12.5" outlineLevelRow="1" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="16384" width="8.66923076923077" style="1"/>
+    <col min="1" max="1" width="5.58461538461538" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8.66923076923077" style="1"/>
+    <col min="3" max="3" width="5.66923076923077" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.08461538461538" style="1" customWidth="1"/>
+    <col min="5" max="5" width="7.75384615384615" style="1" customWidth="1"/>
+    <col min="6" max="6" width="28.8307692307692" style="1" customWidth="1"/>
+    <col min="7" max="8" width="4.5" style="1" customWidth="1"/>
+    <col min="9" max="9" width="4.41538461538462" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.66923076923077" style="1"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="2" spans="1:8">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="142" orientation="portrait"/>
   <headerFooter/>
 </worksheet>
 </file>
@@ -2162,43 +2615,60 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A2:H2"/>
-  <sheetFormatPr defaultColWidth="8.66923076923077" defaultRowHeight="12.5" outlineLevelRow="1" outlineLevelCol="7"/>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultColWidth="8.66923076923077" defaultRowHeight="12.5" outlineLevelRow="2" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="5.58461538461538" style="1" customWidth="1"/>
-    <col min="2" max="2" width="8.66923076923077" style="1"/>
+    <col min="1" max="1" width="25.4153846153846" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.8307692307692" style="1" customWidth="1"/>
     <col min="3" max="3" width="5.66923076923077" style="1" customWidth="1"/>
     <col min="4" max="4" width="7.08461538461538" style="1" customWidth="1"/>
     <col min="5" max="5" width="7.75384615384615" style="1" customWidth="1"/>
-    <col min="6" max="6" width="28.8307692307692" style="1" customWidth="1"/>
+    <col min="6" max="6" width="12.1692307692308" style="1" customWidth="1"/>
     <col min="7" max="8" width="4.5" style="1" customWidth="1"/>
-    <col min="9" max="9" width="4.41538461538462" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.66923076923077" style="1"/>
+    <col min="9" max="16384" width="8.66923076923077" style="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="2"/>
+      <c r="B1" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="2"/>
+    </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="D2" s="2"/>
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="F2" s="2"/>
+      <c r="G2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="2" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="3:3">
+      <c r="C3" s="1" t="s">
+        <v>341</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="142" orientation="portrait"/>
   <headerFooter/>
 </worksheet>
 </file>
@@ -2206,7 +2676,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr defaultColWidth="8.66923076923077" defaultRowHeight="12.5" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="25.5" style="1" customWidth="1"/>
@@ -2221,7 +2691,7 @@
   <sheetData>
     <row r="1" spans="2:2">
       <c r="B1" s="1" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -2237,7 +2707,7 @@
       <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="5" t="s">
         <v>5</v>
       </c>
       <c r="H2" s="1" t="s">
@@ -2246,181 +2716,613 @@
     </row>
     <row r="3" spans="3:3">
       <c r="C3" s="1" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="4:4">
       <c r="D4" s="1" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="3:3">
-      <c r="C6" s="7" t="s">
-        <v>56</v>
+      <c r="C6" s="12" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="3:3">
-      <c r="C7" s="7" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" ht="14.5" spans="3:3">
-      <c r="C9" s="8" t="s">
-        <v>58</v>
+      <c r="C7" s="12" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="9" spans="3:3">
+      <c r="C9" s="13" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="3:5">
-      <c r="C11" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
+      <c r="C11" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
     </row>
     <row r="12" spans="3:5">
-      <c r="C12" s="7"/>
-      <c r="D12" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="E12" s="7"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="E12" s="12"/>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="E13" s="7"/>
+        <v>70</v>
+      </c>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="E13" s="12"/>
     </row>
     <row r="14" spans="3:5">
-      <c r="C14" s="7"/>
-      <c r="D14" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="E14" s="7"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="E14" s="12"/>
     </row>
     <row r="15" spans="3:5">
-      <c r="C15" s="7"/>
-      <c r="D15" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="E15" s="7"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="E15" s="12"/>
     </row>
     <row r="16" spans="3:5">
-      <c r="C16" s="7"/>
-      <c r="D16" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E16" s="7"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="E16" s="12"/>
     </row>
     <row r="17" spans="3:5">
-      <c r="C17" s="7"/>
-      <c r="D17" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="E17" s="7"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E17" s="12"/>
     </row>
     <row r="18" spans="3:5">
-      <c r="C18" s="7"/>
-      <c r="D18" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="E18" s="7"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="E18" s="12"/>
     </row>
     <row r="19" spans="3:5">
-      <c r="C19" s="7"/>
-      <c r="D19" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="E19" s="7"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" s="12"/>
     </row>
     <row r="20" spans="3:5">
-      <c r="C20" s="7"/>
-      <c r="D20" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="E20" s="7"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="E20" s="12"/>
     </row>
     <row r="21" spans="3:5">
-      <c r="C21" s="7"/>
-      <c r="D21" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="E21" s="7"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="E21" s="12"/>
     </row>
     <row r="22" spans="3:5">
-      <c r="C22" s="7"/>
-      <c r="D22" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E22" s="7"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="E22" s="12"/>
     </row>
     <row r="23" spans="3:5">
-      <c r="C23" s="7"/>
-      <c r="D23" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="E23" s="7"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="E23" s="12"/>
     </row>
     <row r="24" spans="3:5">
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
     </row>
     <row r="25" spans="3:3">
-      <c r="C25" s="7" t="s">
-        <v>73</v>
+      <c r="C25" s="12" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="26" spans="3:3">
-      <c r="C26" s="7" t="s">
-        <v>74</v>
+      <c r="C26" s="12" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="27" ht="27" customHeight="1" spans="1:8">
-      <c r="A27" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="B27" s="10"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
-      <c r="H27" s="10"/>
-    </row>
-    <row r="28" spans="3:4">
-      <c r="C28" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="D28" s="7"/>
-    </row>
-    <row r="29" spans="3:4">
-      <c r="C29" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="D29" s="7"/>
-    </row>
-    <row r="30" spans="3:4">
-      <c r="C30" s="7"/>
-      <c r="D30" s="7" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="31" spans="3:4">
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-    </row>
-    <row r="32" spans="1:3">
-      <c r="A32" s="9"/>
-      <c r="B32" s="7"/>
-      <c r="C32" s="7"/>
+      <c r="A27" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="B27" s="15"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="15"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="15"/>
+      <c r="H27" s="15"/>
+    </row>
+    <row r="28" ht="16" customHeight="1" spans="1:8">
+      <c r="A28" s="15"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="15"/>
+    </row>
+    <row r="29" ht="16" customHeight="1" spans="1:8">
+      <c r="A29" s="15"/>
+      <c r="B29" s="15"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="15"/>
+    </row>
+    <row r="30" ht="16" customHeight="1" spans="1:8">
+      <c r="A30" s="15"/>
+      <c r="B30" s="15"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15"/>
+      <c r="H30" s="15"/>
+    </row>
+    <row r="31" ht="16" customHeight="1" spans="1:8">
+      <c r="A31" s="15"/>
+      <c r="B31" s="15"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="15"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15"/>
+      <c r="H31" s="15"/>
+    </row>
+    <row r="32" ht="16" customHeight="1" spans="1:8">
+      <c r="A32" s="15"/>
+      <c r="B32" s="15"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15"/>
+      <c r="H32" s="15"/>
+    </row>
+    <row r="33" ht="16" customHeight="1" spans="1:8">
+      <c r="A33" s="15"/>
+      <c r="B33" s="15"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15"/>
+      <c r="H33" s="15"/>
+    </row>
+    <row r="34" ht="16" customHeight="1" spans="1:8">
+      <c r="A34" s="15"/>
+      <c r="B34" s="15"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="15"/>
+    </row>
+    <row r="35" ht="16" customHeight="1" spans="1:8">
+      <c r="A35" s="15"/>
+      <c r="B35" s="15"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="15"/>
+    </row>
+    <row r="36" ht="16" customHeight="1" spans="1:8">
+      <c r="A36" s="15"/>
+      <c r="B36" s="15"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15"/>
+      <c r="H36" s="15"/>
+    </row>
+    <row r="37" ht="16" customHeight="1" spans="1:8">
+      <c r="A37" s="15"/>
+      <c r="B37" s="15"/>
+      <c r="C37" s="15"/>
+      <c r="D37" s="15"/>
+      <c r="E37" s="15"/>
+      <c r="F37" s="15"/>
+      <c r="G37" s="15"/>
+      <c r="H37" s="15"/>
+    </row>
+    <row r="38" ht="16" customHeight="1" spans="1:8">
+      <c r="A38" s="15"/>
+      <c r="B38" s="15"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="15"/>
+      <c r="E38" s="15"/>
+      <c r="F38" s="15"/>
+      <c r="G38" s="15"/>
+      <c r="H38" s="15"/>
+    </row>
+    <row r="39" ht="16" customHeight="1" spans="1:8">
+      <c r="A39" s="15"/>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="15"/>
+      <c r="F39" s="15"/>
+      <c r="G39" s="15"/>
+      <c r="H39" s="15"/>
+    </row>
+    <row r="40" ht="16" customHeight="1" spans="1:8">
+      <c r="A40" s="15"/>
+      <c r="B40" s="15"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="15"/>
+      <c r="G40" s="15"/>
+      <c r="H40" s="15"/>
+    </row>
+    <row r="41" ht="16" customHeight="1" spans="1:8">
+      <c r="A41" s="15"/>
+      <c r="B41" s="15"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="15"/>
+      <c r="F41" s="15"/>
+      <c r="G41" s="15"/>
+      <c r="H41" s="15"/>
+    </row>
+    <row r="42" ht="16" customHeight="1" spans="1:8">
+      <c r="A42" s="15"/>
+      <c r="B42" s="15"/>
+      <c r="C42" s="15"/>
+      <c r="D42" s="15"/>
+      <c r="E42" s="15"/>
+      <c r="F42" s="15"/>
+      <c r="G42" s="15"/>
+      <c r="H42" s="15"/>
+    </row>
+    <row r="43" ht="16" customHeight="1" spans="1:8">
+      <c r="A43" s="15"/>
+      <c r="B43" s="15"/>
+      <c r="C43" s="15"/>
+      <c r="D43" s="15"/>
+      <c r="E43" s="15"/>
+      <c r="F43" s="15"/>
+      <c r="G43" s="15"/>
+      <c r="H43" s="15"/>
+    </row>
+    <row r="44" ht="16" customHeight="1" spans="1:8">
+      <c r="A44" s="15"/>
+      <c r="B44" s="15"/>
+      <c r="C44" s="15"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="15"/>
+      <c r="F44" s="15"/>
+      <c r="G44" s="15"/>
+      <c r="H44" s="15"/>
+    </row>
+    <row r="45" ht="16" customHeight="1" spans="1:8">
+      <c r="A45" s="15"/>
+      <c r="B45" s="15"/>
+      <c r="C45" s="15"/>
+      <c r="D45" s="15"/>
+      <c r="E45" s="15"/>
+      <c r="F45" s="15"/>
+      <c r="G45" s="15"/>
+      <c r="H45" s="15"/>
+    </row>
+    <row r="46" ht="16" customHeight="1" spans="1:8">
+      <c r="A46" s="15"/>
+      <c r="B46" s="15"/>
+      <c r="C46" s="15"/>
+      <c r="D46" s="15"/>
+      <c r="E46" s="15"/>
+      <c r="F46" s="15"/>
+      <c r="G46" s="15"/>
+      <c r="H46" s="15"/>
+    </row>
+    <row r="47" ht="16" customHeight="1" spans="1:8">
+      <c r="A47" s="15"/>
+      <c r="B47" s="15"/>
+      <c r="C47" s="15"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="15"/>
+      <c r="F47" s="15"/>
+      <c r="G47" s="15"/>
+      <c r="H47" s="15"/>
+    </row>
+    <row r="48" ht="16" customHeight="1" spans="1:8">
+      <c r="A48" s="15"/>
+      <c r="B48" s="15"/>
+      <c r="C48" s="15"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="15"/>
+      <c r="F48" s="15"/>
+      <c r="G48" s="15"/>
+      <c r="H48" s="15"/>
+    </row>
+    <row r="49" ht="16" customHeight="1" spans="1:8">
+      <c r="A49" s="15"/>
+      <c r="B49" s="15"/>
+      <c r="C49" s="15"/>
+      <c r="D49" s="15"/>
+      <c r="E49" s="15"/>
+      <c r="F49" s="15"/>
+      <c r="G49" s="15"/>
+      <c r="H49" s="15"/>
+    </row>
+    <row r="50" ht="16" customHeight="1" spans="1:8">
+      <c r="A50" s="15"/>
+      <c r="B50" s="15"/>
+      <c r="C50" s="15"/>
+      <c r="D50" s="15"/>
+      <c r="E50" s="15"/>
+      <c r="F50" s="15"/>
+      <c r="G50" s="15"/>
+      <c r="H50" s="15"/>
+    </row>
+    <row r="51" ht="16" customHeight="1" spans="1:8">
+      <c r="A51" s="15"/>
+      <c r="B51" s="15"/>
+      <c r="C51" s="15"/>
+      <c r="D51" s="15"/>
+      <c r="E51" s="15"/>
+      <c r="F51" s="15"/>
+      <c r="G51" s="15"/>
+      <c r="H51" s="15"/>
+    </row>
+    <row r="52" ht="16" customHeight="1" spans="1:8">
+      <c r="A52" s="15"/>
+      <c r="B52" s="15"/>
+      <c r="C52" s="15"/>
+      <c r="D52" s="15"/>
+      <c r="E52" s="15"/>
+      <c r="F52" s="15"/>
+      <c r="G52" s="15"/>
+      <c r="H52" s="15"/>
+    </row>
+    <row r="53" ht="16" customHeight="1" spans="1:8">
+      <c r="A53" s="15"/>
+      <c r="B53" s="15"/>
+      <c r="C53" s="15"/>
+      <c r="D53" s="15"/>
+      <c r="E53" s="15"/>
+      <c r="F53" s="15"/>
+      <c r="G53" s="15"/>
+      <c r="H53" s="15"/>
+    </row>
+    <row r="54" ht="16" customHeight="1" spans="1:8">
+      <c r="A54" s="15"/>
+      <c r="B54" s="15"/>
+      <c r="C54" s="15"/>
+      <c r="D54" s="15"/>
+      <c r="E54" s="15"/>
+      <c r="F54" s="15"/>
+      <c r="G54" s="15"/>
+      <c r="H54" s="15"/>
+    </row>
+    <row r="55" ht="16" customHeight="1" spans="1:8">
+      <c r="A55" s="15"/>
+      <c r="B55" s="15"/>
+      <c r="C55" s="15"/>
+      <c r="D55" s="15"/>
+      <c r="E55" s="15"/>
+      <c r="F55" s="15"/>
+      <c r="G55" s="15"/>
+      <c r="H55" s="15"/>
+    </row>
+    <row r="56" ht="16" customHeight="1" spans="1:8">
+      <c r="A56" s="15"/>
+      <c r="B56" s="15"/>
+      <c r="C56" s="15"/>
+      <c r="D56" s="15"/>
+      <c r="E56" s="15"/>
+      <c r="F56" s="15"/>
+      <c r="G56" s="15"/>
+      <c r="H56" s="15"/>
+    </row>
+    <row r="57" ht="16" customHeight="1" spans="1:8">
+      <c r="A57" s="15"/>
+      <c r="B57" s="15"/>
+      <c r="C57" s="15"/>
+      <c r="D57" s="15"/>
+      <c r="E57" s="15"/>
+      <c r="F57" s="15"/>
+      <c r="G57" s="15"/>
+      <c r="H57" s="15"/>
+    </row>
+    <row r="58" ht="16" customHeight="1" spans="1:8">
+      <c r="A58" s="15"/>
+      <c r="B58" s="15"/>
+      <c r="C58" s="15"/>
+      <c r="D58" s="15"/>
+      <c r="E58" s="15"/>
+      <c r="F58" s="15"/>
+      <c r="G58" s="15"/>
+      <c r="H58" s="15"/>
+    </row>
+    <row r="59" ht="16" customHeight="1" spans="1:8">
+      <c r="A59" s="15"/>
+      <c r="B59" s="15"/>
+      <c r="C59" s="15"/>
+      <c r="D59" s="15"/>
+      <c r="E59" s="15"/>
+      <c r="F59" s="15"/>
+      <c r="G59" s="15"/>
+      <c r="H59" s="15"/>
+    </row>
+    <row r="60" ht="16" customHeight="1" spans="1:8">
+      <c r="A60" s="15"/>
+      <c r="B60" s="15"/>
+      <c r="C60" s="15"/>
+      <c r="D60" s="15"/>
+      <c r="E60" s="15"/>
+      <c r="F60" s="15"/>
+      <c r="G60" s="15"/>
+      <c r="H60" s="15"/>
+    </row>
+    <row r="61" ht="16" customHeight="1" spans="1:8">
+      <c r="A61" s="15"/>
+      <c r="B61" s="15"/>
+      <c r="C61" s="15"/>
+      <c r="D61" s="15"/>
+      <c r="E61" s="15"/>
+      <c r="F61" s="15"/>
+      <c r="G61" s="15"/>
+      <c r="H61" s="15"/>
+    </row>
+    <row r="62" ht="16" customHeight="1" spans="1:8">
+      <c r="A62" s="15"/>
+      <c r="B62" s="15"/>
+      <c r="C62" s="15"/>
+      <c r="D62" s="15"/>
+      <c r="E62" s="15"/>
+      <c r="F62" s="15"/>
+      <c r="G62" s="15"/>
+      <c r="H62" s="15"/>
+    </row>
+    <row r="63" ht="16" customHeight="1" spans="1:8">
+      <c r="A63" s="15"/>
+      <c r="B63" s="15"/>
+      <c r="C63" s="15"/>
+      <c r="D63" s="15"/>
+      <c r="E63" s="15"/>
+      <c r="F63" s="15"/>
+      <c r="G63" s="15"/>
+      <c r="H63" s="15"/>
+    </row>
+    <row r="64" ht="16" customHeight="1" spans="1:8">
+      <c r="A64" s="15"/>
+      <c r="B64" s="15"/>
+      <c r="C64" s="15"/>
+      <c r="D64" s="15"/>
+      <c r="E64" s="15"/>
+      <c r="F64" s="15"/>
+      <c r="G64" s="15"/>
+      <c r="H64" s="15"/>
+    </row>
+    <row r="65" ht="16" customHeight="1" spans="1:8">
+      <c r="A65" s="15"/>
+      <c r="B65" s="15"/>
+      <c r="C65" s="15"/>
+      <c r="D65" s="15"/>
+      <c r="E65" s="15"/>
+      <c r="F65" s="15"/>
+      <c r="G65" s="15"/>
+      <c r="H65" s="15"/>
+    </row>
+    <row r="66" ht="16" customHeight="1" spans="1:8">
+      <c r="A66" s="15"/>
+      <c r="B66" s="15"/>
+      <c r="C66" s="15"/>
+      <c r="D66" s="15"/>
+      <c r="E66" s="15"/>
+      <c r="F66" s="15"/>
+      <c r="G66" s="15"/>
+      <c r="H66" s="15"/>
+    </row>
+    <row r="67" ht="16" customHeight="1" spans="1:8">
+      <c r="A67" s="15"/>
+      <c r="B67" s="15"/>
+      <c r="C67" s="15"/>
+      <c r="D67" s="15"/>
+      <c r="E67" s="15"/>
+      <c r="F67" s="15"/>
+      <c r="G67" s="15"/>
+      <c r="H67" s="15"/>
+    </row>
+    <row r="68" ht="16" customHeight="1" spans="1:8">
+      <c r="A68" s="15"/>
+      <c r="B68" s="15"/>
+      <c r="C68" s="15"/>
+      <c r="D68" s="15"/>
+      <c r="E68" s="15"/>
+      <c r="F68" s="15"/>
+      <c r="G68" s="15"/>
+      <c r="H68" s="15"/>
+    </row>
+    <row r="69" ht="16" customHeight="1" spans="1:8">
+      <c r="A69" s="15"/>
+      <c r="B69" s="15"/>
+      <c r="C69" s="15"/>
+      <c r="D69" s="15"/>
+      <c r="E69" s="15"/>
+      <c r="F69" s="15"/>
+      <c r="G69" s="15"/>
+      <c r="H69" s="15"/>
+    </row>
+    <row r="70" spans="3:4">
+      <c r="C70" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="D70" s="12"/>
+    </row>
+    <row r="71" spans="3:4">
+      <c r="C71" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="D71" s="12"/>
+    </row>
+    <row r="72" spans="3:4">
+      <c r="C72" s="12"/>
+      <c r="D72" s="12" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="73" spans="3:4">
+      <c r="C73" s="12"/>
+      <c r="D73" s="12"/>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="B74" s="12"/>
+      <c r="C74" s="12" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75" s="17" t="s">
+        <v>90</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A27:H27"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A74" r:id="rId1" display="https://docs.python.org/3/library/stdtypes.html#binary-sequence-types-bytes-bytearray-memoryview"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
@@ -2429,7 +3331,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:H97"/>
   <sheetFormatPr defaultColWidth="8.66923076923077" defaultRowHeight="12.5" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="24.9153846153846" style="1" customWidth="1"/>
@@ -2444,7 +3346,7 @@
   <sheetData>
     <row r="1" spans="2:2">
       <c r="B1" s="1" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -2460,7 +3362,7 @@
       <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="5" t="s">
         <v>5</v>
       </c>
       <c r="H2" s="1" t="s">
@@ -2469,398 +3371,509 @@
     </row>
     <row r="3" spans="2:7">
       <c r="B3" s="1" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="G3" s="2"/>
+        <v>93</v>
+      </c>
+      <c r="G3" s="5"/>
     </row>
     <row r="4" spans="3:7">
       <c r="C4" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="G4" s="2"/>
+        <v>94</v>
+      </c>
+      <c r="G4" s="5"/>
     </row>
     <row r="5" spans="4:7">
       <c r="D5" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="G5" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="G5" s="5"/>
     </row>
     <row r="6" spans="4:7">
       <c r="D6" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="G6" s="2"/>
+        <v>96</v>
+      </c>
+      <c r="G6" s="5"/>
     </row>
     <row r="7" spans="3:3">
       <c r="C7" s="1" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="4:4">
       <c r="D8" s="1" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="5:5">
       <c r="E9" s="1" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="4:4">
       <c r="D10" s="1" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" spans="4:4">
       <c r="D11" s="1" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="5:5">
       <c r="E12" s="1" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="3:3">
       <c r="C13" s="1" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="4:4">
       <c r="D14" s="1" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" ht="13" spans="2:4">
-      <c r="B15" s="6" t="s">
-        <v>90</v>
+      <c r="B15" s="10" t="s">
+        <v>102</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16" ht="13" spans="2:5">
-      <c r="B16" s="6"/>
+      <c r="B16" s="10"/>
       <c r="C16" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>92</v>
+        <v>103</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="17" ht="13" spans="2:4">
-      <c r="B17" s="6"/>
+      <c r="B17" s="10"/>
       <c r="D17" s="1" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
     </row>
     <row r="18" ht="13" spans="2:2">
-      <c r="B18" s="6"/>
+      <c r="B18" s="10"/>
     </row>
     <row r="19" ht="13" spans="1:3">
       <c r="A19" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="B19" s="6"/>
+        <v>105</v>
+      </c>
+      <c r="B19" s="10"/>
       <c r="C19" s="1" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20" ht="13" spans="2:2">
-      <c r="B20" s="6"/>
+      <c r="B20" s="10"/>
     </row>
     <row r="21" ht="13" spans="2:3">
-      <c r="B21" s="6"/>
+      <c r="B21" s="10"/>
       <c r="C21" s="1" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
     </row>
     <row r="22" ht="13" spans="2:4">
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="D22" s="1" t="s">
-        <v>84</v>
-      </c>
     </row>
     <row r="23" ht="13" spans="2:3">
-      <c r="B23" s="6"/>
+      <c r="B23" s="10"/>
       <c r="C23" s="1" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
     </row>
     <row r="24" ht="13" spans="2:2">
-      <c r="B24" s="6"/>
-    </row>
-    <row r="25" ht="13" spans="2:2">
-      <c r="B25" s="6"/>
+      <c r="B24" s="10"/>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="26" spans="3:5">
       <c r="C26" s="1" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
     </row>
     <row r="27" spans="4:4">
       <c r="D27" s="1" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="28" spans="4:4">
       <c r="D28" s="1" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
     </row>
     <row r="29" spans="4:4">
       <c r="D29" s="1" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
     </row>
     <row r="30" spans="4:4">
       <c r="D30" s="1" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
     </row>
     <row r="32" spans="3:3">
       <c r="C32" s="1" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
     </row>
     <row r="33" spans="3:3">
       <c r="C33" s="1" t="s">
-        <v>102</v>
+        <v>116</v>
       </c>
     </row>
     <row r="34" spans="4:4">
       <c r="D34" s="1" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="35" spans="2:5">
       <c r="B35" s="1" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="36" spans="2:5">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6">
       <c r="B36" s="1" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="37" spans="4:4">
-      <c r="D37" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="38" spans="5:5">
-      <c r="E38" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4">
+        <v>120</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="38" spans="2:4">
+      <c r="B38" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
       <c r="A39" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="D39" s="7" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="40" spans="2:4">
+        <v>127</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="40" spans="2:2">
       <c r="B40" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="41" spans="4:4">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" s="1" t="s">
+        <v>131</v>
+      </c>
       <c r="D41" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="42" spans="3:3">
-      <c r="C42" s="1" t="s">
-        <v>112</v>
+        <v>132</v>
+      </c>
+    </row>
+    <row r="42" spans="2:2">
+      <c r="B42" s="1" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="43" spans="4:4">
       <c r="D43" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5">
-      <c r="A44" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>114</v>
-      </c>
+        <v>134</v>
+      </c>
+    </row>
+    <row r="44" spans="5:5">
       <c r="E44" s="1" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="45" spans="5:5">
-      <c r="E45" s="1" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="46" spans="4:4">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="D45" s="12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="46" spans="2:4">
+      <c r="B46" s="1" t="s">
+        <v>138</v>
+      </c>
       <c r="D46" s="1" t="s">
-        <v>117</v>
+        <v>96</v>
       </c>
     </row>
     <row r="47" spans="4:4">
       <c r="D47" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="48" spans="4:4">
-      <c r="D48" s="1" t="s">
-        <v>87</v>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="48" spans="3:3">
+      <c r="C48" s="1" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="49" spans="4:4">
       <c r="D49" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="51" spans="3:3">
-      <c r="C51" s="1" t="s">
-        <v>119</v>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5">
+      <c r="A50" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="51" spans="5:5">
+      <c r="E51" s="1" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="52" spans="4:4">
       <c r="D52" s="1" t="s">
-        <v>83</v>
+        <v>144</v>
       </c>
     </row>
     <row r="53" spans="4:4">
       <c r="D53" s="1" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
     </row>
     <row r="54" spans="4:4">
       <c r="D54" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="56" spans="3:3">
-      <c r="C56" s="7" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="57" spans="3:4">
-      <c r="C57" s="7"/>
-      <c r="D57" s="7" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="58" spans="3:5">
-      <c r="C58" s="7"/>
-      <c r="E58" s="1" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="59" spans="3:4">
-      <c r="C59" s="7"/>
-      <c r="D59" s="1" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="60" spans="3:5">
-      <c r="C60" s="7"/>
-      <c r="E60" s="1" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="61" spans="3:4">
-      <c r="C61" s="7"/>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="55" spans="4:4">
+      <c r="D55" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="57" spans="2:2">
+      <c r="B57" s="1" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="59" spans="2:2">
+      <c r="B59" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="60" spans="3:3">
+      <c r="C60" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="61" spans="4:4">
       <c r="D61" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="62" spans="3:3">
-      <c r="C62" s="7"/>
-    </row>
-    <row r="63" spans="3:3">
-      <c r="C63" s="7" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="64" spans="4:4">
-      <c r="D64" s="7" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4">
-      <c r="A65" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="D65" s="7" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="66" spans="4:5">
-      <c r="D66" s="7"/>
-      <c r="E66" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="67" spans="4:5">
-      <c r="D67" s="7"/>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="62" spans="4:4">
+      <c r="D62" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="63" spans="4:4">
+      <c r="D63" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="65" spans="3:3">
+      <c r="C65" s="12" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="66" spans="3:4">
+      <c r="C66" s="12"/>
+      <c r="D66" s="12" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="67" spans="3:5">
+      <c r="C67" s="12"/>
       <c r="E67" s="1" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="68" spans="4:4">
-      <c r="D68" s="7" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2">
-      <c r="A70" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="81" spans="3:4">
-      <c r="C81" s="7"/>
-      <c r="D81" s="7"/>
-    </row>
-    <row r="82" spans="3:4">
-      <c r="C82" s="7"/>
-      <c r="D82" s="7"/>
-    </row>
-    <row r="83" spans="3:4">
-      <c r="C83" s="7"/>
-      <c r="D83" s="7"/>
-    </row>
-    <row r="84" spans="3:4">
-      <c r="C84" s="7"/>
-      <c r="D84" s="7"/>
-    </row>
-    <row r="85" spans="3:4">
-      <c r="C85" s="7"/>
-      <c r="D85" s="7"/>
-    </row>
-    <row r="86" spans="4:4">
-      <c r="D86" s="7"/>
-    </row>
-    <row r="87" spans="3:4">
-      <c r="C87" s="7"/>
-      <c r="D87" s="7"/>
+        <v>155</v>
+      </c>
+    </row>
+    <row r="68" spans="3:4">
+      <c r="C68" s="12"/>
+      <c r="D68" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="69" spans="3:5">
+      <c r="C69" s="12"/>
+      <c r="E69" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="70" spans="3:4">
+      <c r="C70" s="12"/>
+      <c r="D70" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="71" spans="3:3">
+      <c r="C71" s="12"/>
+    </row>
+    <row r="72" ht="15.5" spans="1:6">
+      <c r="A72"/>
+      <c r="B72"/>
+      <c r="C72"/>
+      <c r="D72"/>
+      <c r="E72"/>
+      <c r="F72"/>
+    </row>
+    <row r="73" ht="15.5" spans="1:6">
+      <c r="A73"/>
+      <c r="B73"/>
+      <c r="C73"/>
+      <c r="D73"/>
+      <c r="E73"/>
+      <c r="F73"/>
+    </row>
+    <row r="74" ht="15.5" spans="1:6">
+      <c r="A74"/>
+      <c r="B74"/>
+      <c r="C74"/>
+      <c r="D74"/>
+      <c r="E74"/>
+      <c r="F74"/>
+    </row>
+    <row r="75" ht="15.5" spans="1:6">
+      <c r="A75"/>
+      <c r="B75"/>
+      <c r="C75"/>
+      <c r="D75"/>
+      <c r="E75"/>
+      <c r="F75"/>
+    </row>
+    <row r="76" ht="15.5" spans="1:6">
+      <c r="A76"/>
+      <c r="B76"/>
+      <c r="C76"/>
+      <c r="D76"/>
+      <c r="E76"/>
+      <c r="F76"/>
+    </row>
+    <row r="77" ht="15.5" spans="1:6">
+      <c r="A77"/>
+      <c r="B77"/>
+      <c r="C77"/>
+      <c r="D77"/>
+      <c r="E77"/>
+      <c r="F77"/>
+    </row>
+    <row r="78" ht="15.5" spans="1:6">
+      <c r="A78"/>
+      <c r="B78"/>
+      <c r="C78"/>
+      <c r="D78"/>
+      <c r="E78"/>
+      <c r="F78"/>
+    </row>
+    <row r="79" ht="15.5" spans="1:6">
+      <c r="A79"/>
+      <c r="B79"/>
+      <c r="C79"/>
+      <c r="D79"/>
+      <c r="E79"/>
+      <c r="F79"/>
+    </row>
+    <row r="80" ht="15.5" spans="1:6">
+      <c r="A80"/>
+      <c r="B80"/>
+      <c r="C80"/>
+      <c r="D80"/>
+      <c r="E80"/>
+      <c r="F80"/>
+    </row>
+    <row r="91" spans="3:4">
+      <c r="C91" s="12"/>
+      <c r="D91" s="12"/>
+    </row>
+    <row r="92" spans="3:4">
+      <c r="C92" s="12"/>
+      <c r="D92" s="12"/>
+    </row>
+    <row r="93" spans="3:4">
+      <c r="C93" s="12"/>
+      <c r="D93" s="12"/>
+    </row>
+    <row r="94" spans="3:4">
+      <c r="C94" s="12"/>
+      <c r="D94" s="12"/>
+    </row>
+    <row r="95" spans="3:4">
+      <c r="C95" s="12"/>
+      <c r="D95" s="12"/>
+    </row>
+    <row r="96" spans="4:4">
+      <c r="D96" s="12"/>
+    </row>
+    <row r="97" spans="3:4">
+      <c r="C97" s="12"/>
+      <c r="D97" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2872,7 +3885,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr defaultColWidth="8.66923076923077" defaultRowHeight="12.5" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="25.5" style="1" customWidth="1"/>
@@ -2881,13 +3894,14 @@
     <col min="4" max="4" width="3.33076923076923" style="1" customWidth="1"/>
     <col min="5" max="5" width="12.6692307692308" style="1" customWidth="1"/>
     <col min="6" max="6" width="12.1692307692308" style="1" customWidth="1"/>
-    <col min="7" max="8" width="4.5" style="1" customWidth="1"/>
+    <col min="7" max="7" width="4.5" style="8" customWidth="1"/>
+    <col min="8" max="8" width="4.5" style="1" customWidth="1"/>
     <col min="9" max="16384" width="8.66923076923077" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:2">
       <c r="B1" s="1" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -2903,7 +3917,7 @@
       <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="5" t="s">
         <v>5</v>
       </c>
       <c r="H2" s="1" t="s">
@@ -2912,62 +3926,264 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
-        <v>136</v>
+        <v>160</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>137</v>
+        <v>161</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>138</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" spans="2:2">
       <c r="B4" s="1" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" spans="2:2">
       <c r="B5" s="1" t="s">
-        <v>140</v>
+        <v>164</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
-        <v>141</v>
+        <v>167</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>142</v>
+        <v>168</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="1" t="s">
-        <v>143</v>
+        <v>169</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>144</v>
+        <v>170</v>
       </c>
     </row>
     <row r="9" spans="4:4">
       <c r="D9" s="1" t="s">
-        <v>145</v>
+        <v>171</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
-        <v>146</v>
+        <v>172</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>147</v>
+        <v>173</v>
       </c>
     </row>
     <row r="11" spans="4:4">
       <c r="D11" s="1" t="s">
-        <v>148</v>
+        <v>174</v>
       </c>
     </row>
     <row r="12" spans="5:5">
       <c r="E12" s="1" t="s">
-        <v>149</v>
+        <v>175</v>
+      </c>
+    </row>
+    <row r="13" spans="3:3">
+      <c r="C13" s="1" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="9"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="9"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="9"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="F18" s="9"/>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="F19" s="9"/>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="F20" s="9"/>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="9"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="26" spans="2:2">
+      <c r="B26" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="G29" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="32" spans="5:5">
+      <c r="E32" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2">
+      <c r="B34" s="1" t="s">
+        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -2979,413 +4195,668 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H112"/>
   <sheetFormatPr defaultColWidth="8.66923076923077" defaultRowHeight="12.5" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="25.4153846153846" style="3" customWidth="1"/>
-    <col min="2" max="2" width="19.8307692307692" style="3" customWidth="1"/>
-    <col min="3" max="3" width="5.66923076923077" style="3" customWidth="1"/>
-    <col min="4" max="4" width="7.08461538461538" style="3" customWidth="1"/>
-    <col min="5" max="5" width="7.75384615384615" style="3" customWidth="1"/>
-    <col min="6" max="6" width="12.1692307692308" style="3" customWidth="1"/>
-    <col min="7" max="8" width="4.5" style="3" customWidth="1"/>
-    <col min="9" max="16384" width="8.66923076923077" style="3"/>
+    <col min="1" max="1" width="25.4153846153846" style="2" customWidth="1"/>
+    <col min="2" max="2" width="19.8307692307692" style="2" customWidth="1"/>
+    <col min="3" max="3" width="5.66923076923077" style="2" customWidth="1"/>
+    <col min="4" max="4" width="7.08461538461538" style="2" customWidth="1"/>
+    <col min="5" max="5" width="7.75384615384615" style="2" customWidth="1"/>
+    <col min="6" max="6" width="12.1692307692308" style="2" customWidth="1"/>
+    <col min="7" max="7" width="4.5" style="3" customWidth="1"/>
+    <col min="8" max="8" width="4.5" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="8.66923076923077" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:2">
-      <c r="B1" s="3" t="s">
-        <v>150</v>
+      <c r="B1" s="2" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="3:7">
-      <c r="C3" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="G3" s="4"/>
+      <c r="C3" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="G3" s="7"/>
     </row>
     <row r="4" spans="3:7">
-      <c r="C4" s="5"/>
-      <c r="D4" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="E4" s="5"/>
-      <c r="G4" s="4"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="E4" s="6"/>
+      <c r="G4" s="7"/>
     </row>
     <row r="5" spans="3:7">
-      <c r="C5" s="5"/>
-      <c r="D5" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="E5" s="5"/>
-      <c r="G5" s="4"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E5" s="6"/>
+      <c r="G5" s="7"/>
     </row>
     <row r="6" spans="3:7">
-      <c r="C6" s="5"/>
-      <c r="D6" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="E6" s="5"/>
-      <c r="G6" s="4"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="E6" s="6"/>
+      <c r="G6" s="7"/>
     </row>
     <row r="7" spans="3:7">
-      <c r="C7" s="5"/>
-      <c r="D7" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="E7" s="5"/>
-      <c r="G7" s="4"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="E7" s="6"/>
+      <c r="G7" s="7"/>
     </row>
     <row r="8" spans="3:7">
-      <c r="C8" s="5"/>
-      <c r="D8" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="E8" s="5"/>
-      <c r="G8" s="4"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="E8" s="6"/>
+      <c r="G8" s="7"/>
     </row>
     <row r="9" spans="4:7">
-      <c r="D9" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="G9" s="4"/>
+      <c r="D9" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="G9" s="7"/>
     </row>
     <row r="10" spans="4:7">
-      <c r="D10" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="G10" s="4"/>
+      <c r="D10" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="G10" s="7"/>
     </row>
     <row r="11" spans="4:7">
-      <c r="D11" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="G11" s="4"/>
+      <c r="D11" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="G11" s="7"/>
     </row>
     <row r="12" spans="4:7">
       <c r="D12" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="G12" s="4"/>
+        <v>175</v>
+      </c>
+      <c r="G12" s="7"/>
     </row>
     <row r="13" spans="4:7">
-      <c r="D13" s="1"/>
-      <c r="G13" s="4"/>
+      <c r="D13" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="G13" s="7"/>
     </row>
     <row r="14" spans="4:7">
-      <c r="D14" s="1"/>
-      <c r="G14" s="4"/>
+      <c r="D14" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="G14" s="7"/>
     </row>
     <row r="15" spans="4:7">
       <c r="D15" s="1"/>
-      <c r="G15" s="4"/>
-    </row>
-    <row r="16" spans="3:7">
-      <c r="C16" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G16" s="4"/>
+      <c r="G15" s="7"/>
+    </row>
+    <row r="16" spans="4:7">
+      <c r="D16" s="1"/>
+      <c r="G16" s="7"/>
     </row>
     <row r="17" spans="4:7">
-      <c r="D17" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="G17" s="4"/>
+      <c r="D17" s="1"/>
+      <c r="G17" s="7"/>
     </row>
     <row r="18" spans="4:7">
-      <c r="D18" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="G18" s="4"/>
-    </row>
-    <row r="19" spans="7:7">
-      <c r="G19" s="4"/>
-    </row>
-    <row r="20" spans="3:7">
-      <c r="C20" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="D20" s="5"/>
-      <c r="G20" s="4"/>
-    </row>
-    <row r="21" spans="3:7">
-      <c r="C21" s="5"/>
-      <c r="D21" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="G21" s="4"/>
-    </row>
-    <row r="22" spans="3:7">
-      <c r="C22" s="5"/>
-      <c r="D22" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="G22" s="4"/>
-    </row>
-    <row r="23" spans="3:7">
-      <c r="C23" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="D23" s="5"/>
-      <c r="G23" s="4"/>
-    </row>
-    <row r="24" spans="3:7">
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="G24" s="4"/>
-    </row>
-    <row r="25" spans="3:7">
-      <c r="C25" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="D25" s="5"/>
-      <c r="G25" s="4"/>
-    </row>
-    <row r="26" spans="3:7">
-      <c r="C26" s="5"/>
-      <c r="D26" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="G26" s="4"/>
-    </row>
-    <row r="27" spans="7:7">
-      <c r="G27" s="4"/>
-    </row>
-    <row r="28" spans="3:7">
-      <c r="C28" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="G28" s="4"/>
+      <c r="D18" s="1"/>
+      <c r="G18" s="7"/>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="G19" s="7"/>
+    </row>
+    <row r="20" spans="2:7">
+      <c r="B20" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="G20" s="7"/>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="G21" s="7"/>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="G22" s="7"/>
+    </row>
+    <row r="23" spans="4:7">
+      <c r="D23" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="G23" s="7"/>
+    </row>
+    <row r="24" spans="4:7">
+      <c r="D24" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="G24" s="7"/>
+    </row>
+    <row r="25" spans="4:7">
+      <c r="D25" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="G25" s="7"/>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="G26" s="7"/>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="G27" s="7"/>
+    </row>
+    <row r="28" spans="5:7">
+      <c r="E28" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="G28" s="7"/>
     </row>
     <row r="29" spans="4:7">
-      <c r="D29" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="G29" s="4"/>
-    </row>
-    <row r="30" spans="5:7">
-      <c r="E30" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="G30" s="4"/>
-    </row>
-    <row r="31" spans="7:7">
-      <c r="G31" s="4"/>
-    </row>
-    <row r="32" spans="4:7">
-      <c r="D32" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="G32" s="4"/>
-    </row>
-    <row r="33" spans="5:7">
-      <c r="E33" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="G33" s="4"/>
-    </row>
-    <row r="34" spans="5:7">
-      <c r="E34" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="G34" s="4"/>
-    </row>
-    <row r="35" spans="5:7">
-      <c r="E35" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="G35" s="4"/>
+      <c r="D29" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="G29" s="7"/>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="G30" s="7"/>
+    </row>
+    <row r="31" spans="3:7">
+      <c r="C31" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="G31" s="7"/>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="G32" s="7"/>
+    </row>
+    <row r="33" spans="4:7">
+      <c r="D33" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="G33" s="7"/>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="G34" s="7"/>
+    </row>
+    <row r="35" spans="3:7">
+      <c r="C35" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="D35" s="6"/>
+      <c r="G35" s="7"/>
     </row>
     <row r="36" spans="3:7">
-      <c r="C36" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G36" s="4"/>
-    </row>
-    <row r="37" spans="4:7">
-      <c r="D37" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="G37" s="4"/>
-    </row>
-    <row r="38" spans="5:5">
-      <c r="E38" s="3" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="39" spans="4:4">
-      <c r="D39" s="3" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="41" spans="3:3">
-      <c r="C41" s="3" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="42" spans="4:4">
-      <c r="D42" s="3" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="43" spans="3:3">
-      <c r="C43" s="3" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="45" spans="3:3">
-      <c r="C45" s="3" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="47" spans="3:3">
-      <c r="C47" s="3" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="49" spans="3:3">
-      <c r="C49" s="3" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="50" spans="4:5">
-      <c r="D50" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="E50" s="3" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="51" spans="4:4">
-      <c r="D51" s="3" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="53" spans="3:3">
-      <c r="C53" s="3" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="54" spans="4:4">
-      <c r="D54" s="3" t="s">
-        <v>193</v>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="G36" s="7"/>
+    </row>
+    <row r="37" spans="3:7">
+      <c r="C37" s="6"/>
+      <c r="D37" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="G37" s="7"/>
+    </row>
+    <row r="38" spans="3:7">
+      <c r="C38" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="D38" s="6"/>
+      <c r="G38" s="7"/>
+    </row>
+    <row r="39" spans="3:7">
+      <c r="C39" s="6"/>
+      <c r="D39" s="6"/>
+      <c r="G39" s="7"/>
+    </row>
+    <row r="40" spans="3:7">
+      <c r="C40" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="D40" s="6"/>
+      <c r="G40" s="7"/>
+    </row>
+    <row r="41" spans="3:7">
+      <c r="C41" s="6"/>
+      <c r="D41" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="G41" s="7"/>
+    </row>
+    <row r="42" spans="7:7">
+      <c r="G42" s="7"/>
+    </row>
+    <row r="43" spans="3:7">
+      <c r="C43" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="G43" s="7"/>
+    </row>
+    <row r="44" spans="4:7">
+      <c r="D44" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="G44" s="7"/>
+    </row>
+    <row r="45" spans="5:7">
+      <c r="E45" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="G45" s="7"/>
+    </row>
+    <row r="46" spans="7:7">
+      <c r="G46" s="7"/>
+    </row>
+    <row r="47" spans="4:7">
+      <c r="D47" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="G47" s="7"/>
+    </row>
+    <row r="48" spans="5:7">
+      <c r="E48" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="G48" s="7"/>
+    </row>
+    <row r="49" spans="5:7">
+      <c r="E49" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="G49" s="7"/>
+    </row>
+    <row r="50" spans="5:7">
+      <c r="E50" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="G50" s="7"/>
+    </row>
+    <row r="51" spans="1:7">
+      <c r="A51" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="G51" s="7"/>
+    </row>
+    <row r="52" spans="3:7">
+      <c r="C52" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="G52" s="7"/>
+    </row>
+    <row r="53" spans="4:7">
+      <c r="D53" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="G53" s="7"/>
+    </row>
+    <row r="54" spans="5:5">
+      <c r="E54" s="2" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="55" spans="4:4">
-      <c r="D55" s="3" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="56" spans="4:4">
-      <c r="D56" s="3" t="s">
+      <c r="D55" s="2" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="57" spans="2:4">
+      <c r="B57" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="59" spans="3:3">
+      <c r="C59" s="2" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="60" spans="4:4">
+      <c r="D60" s="2" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
+      <c r="A61" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C61" s="2" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="57" spans="4:4">
-      <c r="D57" s="3" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3">
-      <c r="A59" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="C59" s="3" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="61" spans="3:3">
-      <c r="C61" s="3" t="s">
-        <v>199</v>
-      </c>
-    </row>
     <row r="62" spans="4:4">
-      <c r="D62" s="3" t="s">
-        <v>200</v>
+      <c r="D62" s="2" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="63" spans="4:4">
-      <c r="D63" s="3" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3">
-      <c r="A65" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="C65" s="3" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="66" spans="4:4">
-      <c r="D66" s="3" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="67" spans="4:4">
-      <c r="D67" s="3" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="68" spans="4:4">
-      <c r="D68" s="3" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="69" spans="4:4">
-      <c r="D69" s="3" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5">
-      <c r="A70" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="E70" s="3" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5">
-      <c r="A71" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="E71" s="3" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="72" spans="5:5">
-      <c r="E72" s="3" t="s">
-        <v>212</v>
+      <c r="D63" s="2" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="64" spans="3:3">
+      <c r="C64" s="2" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="65" spans="2:4">
+      <c r="B65" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="66" spans="2:2">
+      <c r="B66" s="2" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="67" spans="3:3">
+      <c r="C67" s="2" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="68" spans="4:5">
+      <c r="D68" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4">
+      <c r="A69" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4">
+      <c r="A70" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="71" spans="2:2">
+      <c r="B71" s="2" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="72" spans="2:2">
+      <c r="B72" s="2" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="74" spans="3:3">
+      <c r="C74" s="2" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="75" spans="4:4">
+      <c r="D75" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="76" spans="4:4">
+      <c r="D76" s="2" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="77" spans="4:4">
+      <c r="D77" s="2" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="78" spans="4:4">
+      <c r="D78" s="2" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3">
+      <c r="A79" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="80" spans="2:4">
+      <c r="B80" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3">
+      <c r="A81" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="82" spans="4:4">
+      <c r="D82" s="2" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="83" spans="2:3">
+      <c r="B83" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="84" spans="3:3">
+      <c r="C84" s="2" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3">
+      <c r="A85" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="86" spans="4:4">
+      <c r="D86" s="2" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="87" spans="4:4">
+      <c r="D87" s="2" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3">
+      <c r="A88" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="89" spans="3:3">
+      <c r="C89" s="2" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="90" spans="4:4">
+      <c r="D90" s="2" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="91" spans="4:4">
+      <c r="D91" s="2" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3">
+      <c r="A104" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="105" spans="4:4">
+      <c r="D105" s="2" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="106" spans="4:4">
+      <c r="D106" s="2" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7">
+      <c r="A112" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="G112" s="3">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -3412,7 +4883,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="7:7">
-      <c r="G1" s="2"/>
+      <c r="G1" s="5"/>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="1" t="s">
@@ -3427,7 +4898,7 @@
       <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="5" t="s">
         <v>5</v>
       </c>
       <c r="H2" s="1" t="s">
@@ -3470,7 +4941,7 @@
       <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="5" t="s">
         <v>5</v>
       </c>
       <c r="H2" s="1" t="s">
@@ -3479,37 +4950,39 @@
     </row>
     <row r="3" spans="3:5">
       <c r="C3" s="1" t="s">
-        <v>213</v>
+        <v>332</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>214</v>
+        <v>333</v>
       </c>
     </row>
     <row r="4" spans="3:5">
       <c r="C4" s="1" t="s">
-        <v>215</v>
+        <v>334</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>216</v>
+        <v>335</v>
       </c>
     </row>
     <row r="5" spans="3:5">
       <c r="C5" s="1" t="s">
-        <v>217</v>
+        <v>336</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="6" ht="15.5" spans="3:5">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="6" spans="3:3">
       <c r="C6" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="E6"/>
-    </row>
-    <row r="7" spans="3:3">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="7" spans="3:5">
       <c r="C7" s="1" t="s">
-        <v>220</v>
+        <v>339</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>340</v>
       </c>
     </row>
   </sheetData>

</xml_diff>